<commit_message>
Update BOQ template to match new 2026 single-table BOQ template design (Qty, Made Code, Plan Code, Description, Floor, Area, Material/Colour, Lead Times, Class, Unit Price, Total)
</commit_message>
<xml_diff>
--- a/backend/templates/BOQ/template.xlsx
+++ b/backend/templates/BOQ/template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ Template" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,54 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FF0000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid"/>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +80,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,142 +472,482 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>{{CLIENT_COMPANY}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Bill of Quantity</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{{PROJECT_NAME}}</t>
+          <t>[FIXED]</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Order Reference: {{DOCUMENT_NUMBER}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Project - {{PROJECT_NAME}}</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Order Date: {{DATE}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{{#each items}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Date: {{DATE}}</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{{index}}</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>{{type}}</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>{{description}}</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>{{qty}}</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>{{unitCost}}</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>{{retail}}</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>{{totalRetail}}</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>{{stockStatus}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>One to One Rep : {{ONEONE_REP}}</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Mobile : {{PM_PHONE}}</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Email : {{PM_EMAIL}}</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>{{/each}}</t>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>[TABLE_HEADER]</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Made Code</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Plan Code</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Material/Colour</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Lead Times</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Subtotal:</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>{{SUBTOTAL}}</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>[ITEM]</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.qty}}</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.oneOneCode}}</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.type}}</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.description}}</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.floor}}</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.area}}</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.material/colour}}</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.eta}}</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.class}}</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.retail}}</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>{{item.totalRetail}}</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Discount:</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>{{DISCOUNT_AMOUNT}}</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>[CREDIT_HEADER]</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Made Code</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Plan Code</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>Material/Colour</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Lead Times</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>VAT (15%):</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>{{VAT_AMOUNT}}</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[CREDIT_ITEM]</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.qty}}</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.oneOneCode}}</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.type}}</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.description}}</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.floor}}</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.area}}</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.material/colour}}</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.eta}}</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.class}}</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.retail}}</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>{{item.totalRetail}}</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Grand Total:</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>{{TOTAL_RETAIL}}</t>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>ORDER VALUE (Excl. VAT) : {{SUBTOTAL}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>DISCOUNT : (0% ) {{DISCOUNT_AMOUNT}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>VAT : (15%) {{VAT_AMOUNT}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL VALUE (Incl. VAT) : {{TOTAL_RETAIL}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>70% DEPOSIT INCL VAT : {{DEPOSIT}}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Please see Terms and Conditions which are applicable to all purchases. (Attached)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>* Delivery Fee have not been included in this quote. Should you require 1TO1 Design Studio to deliver, an additional fee will apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>**This quote does not include the LED assembly. If required, please inform the Project Manager and we will revise the quote accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>[FIXED]</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Approval of this Bill of Quantities (BOQ)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="I14:L14"/>
+    <mergeCell ref="B16:L16"/>
+    <mergeCell ref="I15:L15"/>
+    <mergeCell ref="B22:L22"/>
+    <mergeCell ref="B17:L17"/>
+    <mergeCell ref="B18:L18"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>